<commit_message>
docs(docs): CHANGELOG completo del go-live + Excel de egresos (Namecheap)
- CHANGELOG: entrada [1 jul] ampliada con todo el go-live (DMARC, secretos
  rotados, páginas legales, builds Vercel independientes, reset de prod, pie
  de contacto en correos).
- Excel: fila del dominio anota Namecheap (DNS: DMARC/SPF/DKIM/CNAMEs).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Contabilidad_Egresos_AnunciaYA.xlsx
+++ b/docs/Contabilidad_Egresos_AnunciaYA.xlsx
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>MXN</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>ANUAL: renovar cada año o se pierde el dominio. Confirmar costo y fecha de renovación.</t>
+          <t>Registrado en NAMECHEAP (nameservers dns1/dns2.registrar-servers.com); ahí vive el DNS: DMARC, SPF, DKIM y los CNAME de Vercel/SES. ANUAL: renovar cada año o se pierde el dominio. Confirmar costo y fecha exacta de renovación en Namecheap.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(docs): completar Excel de egresos (dominio, Migadu, Gemini)
- Dominio anunciaya.mx (Namecheap): $26.98 1er año / ~$41.98 renovación,
  vence 19-may-2027, tarjeta 3923.
- Migadu: plan Mini $9/mes, renueva día 4, tarjeta 3923.
- Gemini/Coyo: ~$0.07/mes (tokens), hoy cubierto por créditos prepago
  de AI Studio (MXN 189.34); pospago a tarjeta 3923 al agotarse.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Contabilidad_Egresos_AnunciaYA.xlsx
+++ b/docs/Contabilidad_Egresos_AnunciaYA.xlsx
@@ -86,7 +86,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -111,11 +111,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -187,15 +182,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1003,25 +992,21 @@
           <t>Nombre de dominio</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>Registro anual</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Registro anual</t>
-        </is>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Registrado (Namecheap)</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>26.98</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Renovación anual</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>41.98</v>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
@@ -1030,17 +1015,17 @@
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>ANUAL</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
+          <t>ANUAL · renueva 19-may-2027</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>Registrado en NAMECHEAP (nameservers dns1/dns2.registrar-servers.com); ahí vive el DNS: DMARC, SPF, DKIM y los CNAME de Vercel/SES. ANUAL: renovar cada año o se pierde el dominio. Confirmar costo y fecha exacta de renovación en Namecheap.</t>
+          <t>Registrado 18-may-2026 en NAMECHEAP: $26.98 el 1er año (promo; precio normal $41.98) + Free Domain Privacy GRATIS. Renueva ~19-MAY-2027 (~$41.98/año estimado). Ahí vive el DNS (DMARC/SPF/DKIM/CNAMEs Vercel/SES). ANUAL: renovar o se pierde el dominio. OJO: el dominio VIEJO anunciaya.online expira 23-jul-2026 → DEJAR EXPIRAR (ya migrado a .mx).</t>
         </is>
       </c>
     </row>
@@ -1055,25 +1040,21 @@
           <t>Buzones @anunciaya.mx</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="E13" s="14" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Mini ($9/mes)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Mini</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>9</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -1082,17 +1063,17 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>ANUAL</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
+          <t>Mensual · renueva día 4</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>ANUAL. Confirmar plan, costo y fecha de renovación.</t>
+          <t>Plan Mini mensual $9/mes (1000 correos in/día, 100 out/día, 30 GB, dominios/direcciones ilimitados). Renueva mensual (próx. 4-jul-2026). Servidor en Suiza. TIP de ahorro: el plan anual cuesta $90/año (=$7.50/mes, ahorra $18/año) si quieres cambiarlo.</t>
         </is>
       </c>
     </row>
@@ -1107,44 +1088,44 @@
           <t>Asistente Coyo del Home</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Por uso (~$0.07/mes)</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>~$0.07/mes</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Por uso</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Por uso</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>Por uso</t>
-        </is>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>CONFIRMAR</t>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>Por tokens consumidos. Vigilar si Coyo se usa mucho. Confirmar costo.</t>
+          <t>Por tokens (gemini 2.5 flash). HOY ~$0.07 USD/mes (centavos, sin usuarios; forecast del mes = $0). Se paga PRIMERO con créditos PREPAGO de AI Studio (MXN 189.34 restantes de MXN 200 agregados 31-may; vencen ~1 año) → $0 de la tarjeta hasta agotarlos. Al agotarse, cobra pospago a la tarjeta 3923. Vigilar si Coyo se usa mucho en la beta.</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1160,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>ESCENARIO A — HOY (fase de pruebas, sin usuarios)</t>
         </is>
@@ -1263,19 +1244,19 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>TOTAL HOY (USD/mes)</t>
         </is>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="16">
         <f>SUM(B5:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="19" t="n"/>
+      <c r="C9" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>ESCENARIO B — AL PROMOVER (decisión: subir antes de abrir a usuarios reales)</t>
         </is>
@@ -1359,16 +1340,16 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>TOTAL AL PROMOVER (USD/mes)</t>
         </is>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="19">
         <f>SUM(B14:B17)</f>
         <v/>
       </c>
-      <c r="C18" s="19" t="n"/>
+      <c r="C18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1378,9 +1359,9 @@
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>ADEMÁS (no fijos): Stripe (comisiones por cobro ~3.6%+$3+IVA) · AWS SES (~$0.10/1000 correos) · Cloudflare R2 (10GB gratis, luego ~$0.015/GB) · ANUALES: dominio anunciaya.mx y correo Migadu (¡vigilar fecha de renovación!). Servicios en USD: multiplicar por tipo de cambio del día para tu contabilidad en MXN.</t>
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t>ADEMÁS: Stripe (comisiones por cobro ~3.6%+$3+IVA) · AWS SES (~$0.10/1000 correos) · Cloudflare R2 (10GB gratis, luego ~$0.015/GB) · Gemini/Coyo (~$0.07/mes, hoy cubierto por créditos prepago de AI Studio). Correo MENSUAL: Migadu $9/mes (renueva día 4). ANUAL: dominio anunciaya.mx ~$42/año (renueva 19-may-2027; NO renovar el viejo anunciaya.online, expira 23-jul-2026). Servicios en USD: multiplicar por tipo de cambio para tu contabilidad en MXN.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
@ docs(egresos): agrega herramientas de trabajo/contenido al Excel
CapCut Pro, Google AI Pro (Google One), Canva Business y Claude Plan Max
en una sección aparte (marca "trabajo", azul) + bloque de resumen en la
Hoja 2 con costo/moneda/frecuencia/tarjeta y subtotales por moneda
(935 MXN/mes + 100 USD/mes, todo con la tarjeta …3923).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/docs/Contabilidad_Egresos_AnunciaYA.xlsx
+++ b/docs/Contabilidad_Egresos_AnunciaYA.xlsx
@@ -145,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,6 +182,15 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -191,6 +200,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -556,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -581,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2 jul 2026 · 'Plan al promover' = decisión tomada antes de salir a promocionar · Amarillo = por confirmar · Rojo = subir ANTES de promover · Verde = reaccionar/ok</t>
+          <t>Actualizado 2 jul 2026 · 'Plan al promover' = decisión antes de promocionar · Amarillo = por confirmar · Rojo = subir ANTES de promover · Verde = ok/reaccionar · Azul = herramienta de trabajo/contenido</t>
         </is>
       </c>
     </row>
@@ -1126,6 +1136,198 @@
       <c r="J14" s="9" t="inlineStr">
         <is>
           <t>Por tokens (gemini 2.5 flash). HOY ~$0.07 USD/mes (centavos, sin usuarios; forecast del mes = $0). Se paga PRIMERO con créditos PREPAGO de AI Studio (MXN 189.34 restantes de MXN 200 agregados 31-may; vencen ~1 año) → $0 de la tarjeta hasta agotarlos. Al agotarse, cobra pospago a la tarjeta 3923. Vigilar si Coyo se usa mucho en la beta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="54" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>CapCut Pro</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>[TRABAJO] Edición de video</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>330</v>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>330</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Mensual · renueva 19-jul</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>HERRAMIENTA DE TRABAJO/CONTENIDO. CapCut Pro $330 MXN/mes (renueva 19-jul-2026): 1 TB de almacenamiento + 1250 créditos/mes + activos y plantillas de pago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Pro (Google One)</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>[TRABAJO] IA para imágenes/contenido</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Pro 5 TB</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>395</v>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Pro 5 TB</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>395</v>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Mensual · renueva día 30</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>HERRAMIENTA DE TRABAJO/CONTENIDO. Google AI Pro (Google One) $395 MXN/mes: 5 TB + Gemini avanzado (4x) + Google Flow/modelos creativos + NotebookLM + Gemini en Gmail/Docs. Renueva día 30 (el 1er mes fue $40 de promo). NO confundir con la Gemini API de Coyo (esa es aparte, por tokens). TIP: plan anual $3,949 MXN/año (ahorra 16%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Canva Business</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>[TRABAJO] Diseño gráfico/contenido</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>210</v>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>210</v>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Mensual · renueva 13-jul</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>HERRAMIENTA DE TRABAJO/CONTENIDO. Canva Business $210 MXN/mes (renovación automática, próx. 13-jul-2026): 1 integrante. TIP: cambiar a anual ahorra 16%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Claude (Plan Max)</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>[TRABAJO] Asistente de desarrollo/IA</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Max (5x Pro)</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Max (5x Pro)</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Mensual · renueva 12-jul</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>HERRAMIENTA DE TRABAJO/CONTENIDO. Claude Plan Max $100 USD/mes (5x uso vs Pro; renovación automática, próx. 12-jul-2026). Se paga vía Link by Stripe con la tarjeta 3923. OJO: única herramienta de contenido en USD (las otras 3 son MXN).</t>
         </is>
       </c>
     </row>
@@ -1144,12 +1346,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1160,7 +1364,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>ESCENARIO A — HOY (fase de pruebas, sin usuarios)</t>
         </is>
@@ -1244,19 +1448,19 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>TOTAL HOY (USD/mes)</t>
         </is>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="19">
         <f>SUM(B5:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="17" t="n"/>
+      <c r="C9" s="20" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>ESCENARIO B — AL PROMOVER (decisión: subir antes de abrir a usuarios reales)</t>
         </is>
@@ -1340,16 +1544,16 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>TOTAL AL PROMOVER (USD/mes)</t>
         </is>
       </c>
-      <c r="B18" s="19">
+      <c r="B18" s="22">
         <f>SUM(B14:B17)</f>
         <v/>
       </c>
-      <c r="C18" s="17" t="n"/>
+      <c r="C18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1359,16 +1563,186 @@
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="23" t="inlineStr">
         <is>
           <t>ADEMÁS: Stripe (comisiones por cobro ~3.6%+$3+IVA) · AWS SES (~$0.10/1000 correos) · Cloudflare R2 (10GB gratis, luego ~$0.015/GB) · Gemini/Coyo (~$0.07/mes, hoy cubierto por créditos prepago de AI Studio). Correo MENSUAL: Migadu $9/mes (renueva día 4). ANUAL: dominio anunciaya.mx ~$42/año (renueva 19-may-2027; NO renovar el viejo anunciaya.online, expira 23-jul-2026). Servicios en USD: multiplicar por tipo de cambio para tu contabilidad en MXN.</t>
         </is>
       </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>HERRAMIENTAS DE TRABAJO / CONTENIDO (marketing — no es infra de la app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Herramienta</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Moneda</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Frecuencia</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>CapCut Pro</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>330</v>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Mensual · renueva 19-jul</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Google AI Pro (Google One)</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>395</v>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Mensual · renueva día 30</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Canva Business</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>210</v>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Mensual · renueva 13-jul</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Claude (Plan Max)</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Mensual · renueva 12-jul</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>MasterCard …3923</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>Subtotal contenido (MXN/mes)</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>SUM(B25:B27)</f>
+        <v/>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="n"/>
+      <c r="E29" s="20" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Subtotal contenido (USD/mes)</t>
+        </is>
+      </c>
+      <c r="B30" s="19">
+        <f>B28</f>
+        <v/>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A21:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(sentry): agregar Sentry al control de egresos (infra + resumen mensual)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Contabilidad_Egresos_AnunciaYA.xlsx
+++ b/docs/Contabilidad_Egresos_AnunciaYA.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1328,6 +1328,54 @@
       <c r="J18" s="9" t="inlineStr">
         <is>
           <t>HERRAMIENTA DE TRABAJO/CONTENIDO. Claude Plan Max $100 USD/mes (5x uso vs Pro; renovación automática, próx. 12-jul-2026). Se paga vía Link by Stripe con la tarjeta 3923. OJO: única herramienta de contenido en USD (las otras 3 son MXN).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Sentry (Error tracking)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Monitoreo de errores en prod (frontend + backend)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Developer (gratis)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Developer (gratis) - se mantiene; subir a Team solo si supera 5k errores/mes</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Mensual</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>N/A (gratis)</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>HECHO 8-jul: error tracking en api/web/admin, SOLO en prod. Gratis = 5,000 errores/mes, 1 usuario, sin tarjeta. Org anunciaya en sentry.io, 3 proyectos (api/web/admin). Alertas por correo a admin@anunciaya.mx. REACCIONAR: si en la beta se pasan los ~5k errores/mes, subir a Team (~$26-29/mes, por confirmar). Ver docs/DESPLIEGUE_PRODUCCION.md.</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1613,7 @@
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>ADEMÁS: Stripe (comisiones por cobro ~3.6%+$3+IVA) · AWS SES (~$0.10/1000 correos) · Cloudflare R2 (10GB gratis, luego ~$0.015/GB) · Gemini/Coyo (~$0.07/mes, hoy cubierto por créditos prepago de AI Studio). Correo MENSUAL: Migadu $9/mes (renueva día 4). ANUAL: dominio anunciaya.mx ~$42/año (renueva 19-may-2027; NO renovar el viejo anunciaya.online, expira 23-jul-2026). Servicios en USD: multiplicar por tipo de cambio para tu contabilidad en MXN.</t>
+          <t>ADEMÁS: Stripe (comisiones por cobro ~3.6%+$3+IVA) · AWS SES (~$0.10/1000 correos) · Cloudflare R2 (10GB gratis, luego ~$0.015/GB) · Gemini/Coyo (~$0.07/mes, hoy cubierto por créditos prepago de AI Studio) · Sentry (error tracking: gratis hasta 5,000 errores/mes; sube a Team ~$26-29/mes solo si supera la cuota). Correo MENSUAL: Migadu $9/mes (renueva día 4). ANUAL: dominio anunciaya.mx ~$42/año (renueva 19-may-2027; NO renovar el viejo anunciaya.online, expira 23-jul-2026). Servicios en USD: multiplicar por tipo de cambio para tu contabilidad en MXN.</t>
         </is>
       </c>
     </row>

</xml_diff>